<commit_message>
No major change, formatting only
</commit_message>
<xml_diff>
--- a/inputs/storage_elevation_table.xlsx
+++ b/inputs/storage_elevation_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\calsim_gits\eis-appendix-gen_upd\eis-appendix-generation\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF324794-CB24-440D-98C9-DCAD92CD021F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C2FA3C-0179-46EC-9FE4-2A215341EC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{B92DCBF1-963B-4AC9-BF86-DA13944A9E5F}"/>
+    <workbookView xWindow="-25020" yWindow="1095" windowWidth="23010" windowHeight="12360" xr2:uid="{B92DCBF1-963B-4AC9-BF86-DA13944A9E5F}"/>
   </bookViews>
   <sheets>
     <sheet name="res_info" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Added max storage elevation relationship in storage-elevation table. Based on the res_info.table tables in the Sac LTO Calsim files. Minor modifications to storage-elevation related functions for throwing descriptive errors and fixing San Luis field name
</commit_message>
<xml_diff>
--- a/inputs/storage_elevation_table.xlsx
+++ b/inputs/storage_elevation_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\calsim_gits\eis-appendix-gen_upd\eis-appendix-generation\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C2FA3C-0179-46EC-9FE4-2A215341EC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E474C655-304F-42A6-9439-BC407C482718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25020" yWindow="1095" windowWidth="23010" windowHeight="12360" xr2:uid="{B92DCBF1-963B-4AC9-BF86-DA13944A9E5F}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{B92DCBF1-963B-4AC9-BF86-DA13944A9E5F}"/>
   </bookViews>
   <sheets>
     <sheet name="res_info" sheetId="1" r:id="rId1"/>
@@ -265,12 +265,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -285,8 +297,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -621,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9390FDB4-AB03-46CA-ADC9-91201B613C80}">
-  <dimension ref="A1:F1008"/>
+  <dimension ref="A1:L1009"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" customWidth="1"/>
@@ -2717,19 +2731,19 @@
       <c r="A105">
         <v>11</v>
       </c>
-      <c r="B105">
-        <v>0</v>
-      </c>
-      <c r="C105">
-        <v>0</v>
-      </c>
-      <c r="D105">
-        <v>0</v>
-      </c>
-      <c r="E105">
-        <v>0</v>
-      </c>
-      <c r="F105">
+      <c r="B105" s="1">
+        <v>0</v>
+      </c>
+      <c r="C105" s="1">
+        <v>0</v>
+      </c>
+      <c r="D105" s="1">
+        <v>0</v>
+      </c>
+      <c r="E105" s="1">
+        <v>0</v>
+      </c>
+      <c r="F105" s="1">
         <v>4.4389999999999999E-2</v>
       </c>
     </row>
@@ -2737,19 +2751,19 @@
       <c r="A106">
         <v>11</v>
       </c>
-      <c r="B106">
+      <c r="B106" s="1">
         <v>37980</v>
       </c>
-      <c r="C106">
+      <c r="C106" s="1">
         <v>1686</v>
       </c>
-      <c r="D106">
+      <c r="D106" s="1">
         <v>14376</v>
       </c>
-      <c r="E106">
+      <c r="E106" s="1">
         <v>326.2</v>
       </c>
-      <c r="F106">
+      <c r="F106" s="1">
         <v>1.304E-2</v>
       </c>
     </row>
@@ -2757,19 +2771,19 @@
       <c r="A107">
         <v>11</v>
       </c>
-      <c r="B107">
+      <c r="B107" s="1">
         <v>142500</v>
       </c>
-      <c r="C107">
+      <c r="C107" s="1">
         <v>3049</v>
       </c>
-      <c r="D107">
+      <c r="D107" s="1">
         <v>14376</v>
       </c>
-      <c r="E107">
+      <c r="E107" s="1">
         <v>369.2</v>
       </c>
-      <c r="F107">
+      <c r="F107" s="1">
         <v>6.7799999999999996E-3</v>
       </c>
     </row>
@@ -2777,19 +2791,19 @@
       <c r="A108">
         <v>11</v>
       </c>
-      <c r="B108">
+      <c r="B108" s="1">
         <v>247000</v>
       </c>
-      <c r="C108">
+      <c r="C108" s="1">
         <v>3757</v>
       </c>
-      <c r="D108">
+      <c r="D108" s="1">
         <v>14376</v>
       </c>
-      <c r="E108">
+      <c r="E108" s="1">
         <v>399.6</v>
       </c>
-      <c r="F108">
+      <c r="F108" s="1">
         <v>5.0299999999999997E-3</v>
       </c>
     </row>
@@ -2797,19 +2811,19 @@
       <c r="A109">
         <v>11</v>
       </c>
-      <c r="B109">
+      <c r="B109" s="1">
         <v>356250</v>
       </c>
-      <c r="C109">
+      <c r="C109" s="1">
         <v>4307</v>
       </c>
-      <c r="D109">
+      <c r="D109" s="1">
         <v>14376</v>
       </c>
-      <c r="E109">
+      <c r="E109" s="1">
         <v>426.6</v>
       </c>
-      <c r="F109">
+      <c r="F109" s="1">
         <v>3.6900000000000001E-3</v>
       </c>
     </row>
@@ -2817,19 +2831,19 @@
       <c r="A110">
         <v>11</v>
       </c>
-      <c r="B110">
+      <c r="B110" s="1">
         <v>475000</v>
       </c>
-      <c r="C110">
+      <c r="C110" s="1">
         <v>4745</v>
       </c>
-      <c r="D110">
+      <c r="D110" s="1">
         <v>14376</v>
       </c>
-      <c r="E110">
+      <c r="E110" s="1">
         <v>452.8</v>
       </c>
-      <c r="F110">
+      <c r="F110" s="1">
         <v>2.96E-3</v>
       </c>
     </row>
@@ -2837,19 +2851,19 @@
       <c r="A111">
         <v>11</v>
       </c>
-      <c r="B111">
+      <c r="B111" s="1">
         <v>665000</v>
       </c>
-      <c r="C111">
+      <c r="C111" s="1">
         <v>5307</v>
       </c>
-      <c r="D111">
+      <c r="D111" s="1">
         <v>14376</v>
       </c>
-      <c r="E111">
+      <c r="E111" s="1">
         <v>490.5</v>
       </c>
-      <c r="F111">
+      <c r="F111" s="1">
         <v>2.5500000000000002E-3</v>
       </c>
     </row>
@@ -2857,263 +2871,463 @@
       <c r="A112">
         <v>11</v>
       </c>
-      <c r="B112">
+      <c r="B112" s="1">
         <v>807500</v>
       </c>
-      <c r="C112">
+      <c r="C112" s="1">
         <v>5670</v>
       </c>
-      <c r="D112">
+      <c r="D112" s="1">
         <v>14376</v>
       </c>
-      <c r="E112">
+      <c r="E112" s="1">
         <v>516.4</v>
       </c>
-      <c r="F112">
+      <c r="F112" s="1">
         <v>2.3900000000000002E-3</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>11</v>
       </c>
-      <c r="B113">
+      <c r="B113" s="1">
         <v>902500</v>
       </c>
-      <c r="C113">
+      <c r="C113" s="1">
         <v>5897</v>
       </c>
-      <c r="D113">
+      <c r="D113" s="1">
         <v>14376</v>
       </c>
-      <c r="E113">
+      <c r="E113" s="1">
         <v>532.79999999999995</v>
       </c>
-      <c r="F113">
+      <c r="F113" s="1">
         <v>2.16E-3</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>11</v>
       </c>
-      <c r="B114">
+      <c r="B114" s="1">
         <v>998000</v>
       </c>
-      <c r="C114">
+      <c r="C114" s="1">
         <v>6103</v>
       </c>
-      <c r="D114">
+      <c r="D114" s="1">
         <v>14376</v>
       </c>
-      <c r="E114">
+      <c r="E114" s="1">
         <v>548.70000000000005</v>
       </c>
-      <c r="F114">
+      <c r="F114" s="1">
         <v>2.16E-3</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>12</v>
       </c>
-      <c r="B115">
-        <v>0</v>
-      </c>
-      <c r="C115">
-        <v>0</v>
-      </c>
-      <c r="D115">
-        <v>0</v>
-      </c>
-      <c r="E115">
-        <v>0</v>
-      </c>
-      <c r="F115">
+      <c r="B115" s="2">
+        <v>0</v>
+      </c>
+      <c r="C115" s="2">
+        <v>0</v>
+      </c>
+      <c r="D115" s="2">
+        <v>0</v>
+      </c>
+      <c r="E115" s="2">
+        <v>0</v>
+      </c>
+      <c r="F115" s="2">
         <v>4.4380000000000003E-2</v>
       </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H115">
+        <f>AVERAGE(B115,B105)</f>
+        <v>0</v>
+      </c>
+      <c r="I115">
+        <f t="shared" ref="I115:M124" si="0">AVERAGE(C115,C105)</f>
+        <v>0</v>
+      </c>
+      <c r="J115">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K115">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L115">
+        <f t="shared" si="0"/>
+        <v>4.4385000000000001E-2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>12</v>
       </c>
-      <c r="B116">
+      <c r="B116" s="2">
         <v>42000</v>
       </c>
-      <c r="C116">
+      <c r="C116" s="2">
         <v>1864</v>
       </c>
-      <c r="D116">
+      <c r="D116" s="2">
         <v>14376</v>
       </c>
-      <c r="E116">
+      <c r="E116" s="2">
         <v>326.2</v>
       </c>
-      <c r="F116">
+      <c r="F116" s="2">
         <v>1.303E-2</v>
       </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H116">
+        <f t="shared" ref="H116:H124" si="1">AVERAGE(B116,B106)</f>
+        <v>39990</v>
+      </c>
+      <c r="I116">
+        <f t="shared" si="0"/>
+        <v>1775</v>
+      </c>
+      <c r="J116">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K116">
+        <f t="shared" si="0"/>
+        <v>326.2</v>
+      </c>
+      <c r="L116">
+        <f t="shared" si="0"/>
+        <v>1.3035E-2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>12</v>
       </c>
-      <c r="B117">
+      <c r="B117" s="2">
         <v>157500</v>
       </c>
-      <c r="C117">
+      <c r="C117" s="2">
         <v>3369</v>
       </c>
-      <c r="D117">
+      <c r="D117" s="2">
         <v>14376</v>
       </c>
-      <c r="E117">
+      <c r="E117" s="2">
         <v>369.2</v>
       </c>
-      <c r="F117">
+      <c r="F117" s="2">
         <v>6.79E-3</v>
       </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H117">
+        <f t="shared" si="1"/>
+        <v>150000</v>
+      </c>
+      <c r="I117">
+        <f t="shared" si="0"/>
+        <v>3209</v>
+      </c>
+      <c r="J117">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K117">
+        <f t="shared" si="0"/>
+        <v>369.2</v>
+      </c>
+      <c r="L117">
+        <f t="shared" si="0"/>
+        <v>6.7849999999999994E-3</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>12</v>
       </c>
-      <c r="B118">
+      <c r="B118" s="2">
         <v>273000</v>
       </c>
-      <c r="C118">
+      <c r="C118" s="2">
         <v>4153</v>
       </c>
-      <c r="D118">
+      <c r="D118" s="2">
         <v>14376</v>
       </c>
-      <c r="E118">
+      <c r="E118" s="2">
         <v>399.6</v>
       </c>
-      <c r="F118">
+      <c r="F118" s="2">
         <v>5.0400000000000002E-3</v>
       </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H118">
+        <f t="shared" si="1"/>
+        <v>260000</v>
+      </c>
+      <c r="I118">
+        <f t="shared" si="0"/>
+        <v>3955</v>
+      </c>
+      <c r="J118">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K118">
+        <f t="shared" si="0"/>
+        <v>399.6</v>
+      </c>
+      <c r="L118">
+        <f t="shared" si="0"/>
+        <v>5.0349999999999995E-3</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>12</v>
       </c>
-      <c r="B119">
+      <c r="B119" s="2">
         <v>393750</v>
       </c>
-      <c r="C119">
+      <c r="C119" s="2">
         <v>4761</v>
       </c>
-      <c r="D119">
+      <c r="D119" s="2">
         <v>14376</v>
       </c>
-      <c r="E119">
+      <c r="E119" s="2">
         <v>426.6</v>
       </c>
-      <c r="F119">
+      <c r="F119" s="2">
         <v>3.6900000000000001E-3</v>
       </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H119">
+        <f t="shared" si="1"/>
+        <v>375000</v>
+      </c>
+      <c r="I119">
+        <f t="shared" si="0"/>
+        <v>4534</v>
+      </c>
+      <c r="J119">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K119">
+        <f t="shared" si="0"/>
+        <v>426.6</v>
+      </c>
+      <c r="L119">
+        <f t="shared" si="0"/>
+        <v>3.6900000000000001E-3</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>12</v>
       </c>
-      <c r="B120">
+      <c r="B120" s="2">
         <v>525000</v>
       </c>
-      <c r="C120">
+      <c r="C120" s="2">
         <v>5245</v>
       </c>
-      <c r="D120">
+      <c r="D120" s="2">
         <v>14376</v>
       </c>
-      <c r="E120">
+      <c r="E120" s="2">
         <v>452.8</v>
       </c>
-      <c r="F120">
+      <c r="F120" s="2">
         <v>2.9499999999999999E-3</v>
       </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H120">
+        <f t="shared" si="1"/>
+        <v>500000</v>
+      </c>
+      <c r="I120">
+        <f t="shared" si="0"/>
+        <v>4995</v>
+      </c>
+      <c r="J120">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K120">
+        <f t="shared" si="0"/>
+        <v>452.8</v>
+      </c>
+      <c r="L120">
+        <f t="shared" si="0"/>
+        <v>2.9550000000000002E-3</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>12</v>
       </c>
-      <c r="B121">
+      <c r="B121" s="2">
         <v>735000</v>
       </c>
-      <c r="C121">
+      <c r="C121" s="2">
         <v>5865</v>
       </c>
-      <c r="D121">
+      <c r="D121" s="2">
         <v>14376</v>
       </c>
-      <c r="E121">
+      <c r="E121" s="2">
         <v>490.5</v>
       </c>
-      <c r="F121">
+      <c r="F121" s="2">
         <v>2.5500000000000002E-3</v>
       </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H121">
+        <f t="shared" si="1"/>
+        <v>700000</v>
+      </c>
+      <c r="I121">
+        <f t="shared" si="0"/>
+        <v>5586</v>
+      </c>
+      <c r="J121">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K121">
+        <f t="shared" si="0"/>
+        <v>490.5</v>
+      </c>
+      <c r="L121">
+        <f t="shared" si="0"/>
+        <v>2.5500000000000002E-3</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>12</v>
       </c>
-      <c r="B122">
+      <c r="B122" s="2">
         <v>892500</v>
       </c>
-      <c r="C122">
+      <c r="C122" s="2">
         <v>6266</v>
       </c>
-      <c r="D122">
+      <c r="D122" s="2">
         <v>14376</v>
       </c>
-      <c r="E122">
+      <c r="E122" s="2">
         <v>516.4</v>
       </c>
-      <c r="F122">
+      <c r="F122" s="2">
         <v>2.3999999999999998E-3</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H122">
+        <f t="shared" si="1"/>
+        <v>850000</v>
+      </c>
+      <c r="I122">
+        <f t="shared" si="0"/>
+        <v>5968</v>
+      </c>
+      <c r="J122">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K122">
+        <f t="shared" si="0"/>
+        <v>516.4</v>
+      </c>
+      <c r="L122">
+        <f t="shared" si="0"/>
+        <v>2.395E-3</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>12</v>
       </c>
-      <c r="B123">
+      <c r="B123" s="2">
         <v>997500</v>
       </c>
-      <c r="C123">
+      <c r="C123" s="2">
         <v>6518</v>
       </c>
-      <c r="D123">
+      <c r="D123" s="2">
         <v>14376</v>
       </c>
-      <c r="E123">
+      <c r="E123" s="2">
         <v>532.79999999999995</v>
       </c>
-      <c r="F123">
+      <c r="F123" s="2">
         <v>2.1700000000000001E-3</v>
       </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H123">
+        <f t="shared" si="1"/>
+        <v>950000</v>
+      </c>
+      <c r="I123">
+        <f t="shared" si="0"/>
+        <v>6207.5</v>
+      </c>
+      <c r="J123">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K123">
+        <f t="shared" si="0"/>
+        <v>532.79999999999995</v>
+      </c>
+      <c r="L123">
+        <f t="shared" si="0"/>
+        <v>2.1650000000000003E-3</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>12</v>
       </c>
-      <c r="B124">
+      <c r="B124" s="2">
         <v>1102000</v>
       </c>
-      <c r="C124">
+      <c r="C124" s="2">
         <v>6745</v>
       </c>
-      <c r="D124">
+      <c r="D124" s="2">
         <v>14376</v>
       </c>
-      <c r="E124">
+      <c r="E124" s="2">
         <v>548.70000000000005</v>
       </c>
-      <c r="F124">
+      <c r="F124" s="2">
         <v>2.1700000000000001E-3</v>
       </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H124">
+        <f t="shared" si="1"/>
+        <v>1050000</v>
+      </c>
+      <c r="I124">
+        <f t="shared" si="0"/>
+        <v>6424</v>
+      </c>
+      <c r="J124">
+        <f t="shared" si="0"/>
+        <v>14376</v>
+      </c>
+      <c r="K124">
+        <f t="shared" si="0"/>
+        <v>548.70000000000005</v>
+      </c>
+      <c r="L124">
+        <f t="shared" si="0"/>
+        <v>2.1650000000000003E-3</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>13</v>
       </c>
@@ -3133,7 +3347,7 @@
         <v>4.4359999999999997E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>13</v>
       </c>
@@ -3153,7 +3367,7 @@
         <v>1.303E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>13</v>
       </c>
@@ -3173,7 +3387,7 @@
         <v>6.79E-3</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>13</v>
       </c>
@@ -20701,6 +20915,18 @@
       </c>
       <c r="E1008">
         <v>548.70000000000005</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1009">
+        <v>999</v>
+      </c>
+      <c r="B1009">
+        <f>1200000*2</f>
+        <v>2400000</v>
+      </c>
+      <c r="E1009">
+        <v>581.20000000000005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>